<commit_message>
added new sweeps buckets
</commit_message>
<xml_diff>
--- a/site-src/examples/owlplanner/HFP_alex+jamie.xlsx
+++ b/site-src/examples/owlplanner/HFP_alex+jamie.xlsx
@@ -497,22 +497,15 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>6500</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>0</v>
       </c>
@@ -521,22 +514,15 @@
       <c r="A3" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>6500</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>0</v>
       </c>
@@ -545,22 +531,15 @@
       <c r="A4" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>7000</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>0</v>
       </c>
@@ -578,15 +557,9 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>7000</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>0</v>
       </c>
@@ -604,17 +577,12 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>7000</v>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
         <v>20000</v>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>0</v>
       </c>
@@ -632,15 +600,9 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>15000</v>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>4000</v>
       </c>
@@ -658,15 +620,9 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>15000</v>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>4000</v>
       </c>
@@ -684,15 +640,9 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
         <v>50000</v>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>0</v>
       </c>
@@ -701,22 +651,15 @@
       <c r="A10" t="n">
         <v>2029</v>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
         <v>50000</v>
       </c>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>0</v>
       </c>
@@ -725,20 +668,12 @@
       <c r="A11" t="n">
         <v>2030</v>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>0</v>
       </c>
@@ -747,20 +682,12 @@
       <c r="A12" t="n">
         <v>2031</v>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>0</v>
       </c>
@@ -769,20 +696,12 @@
       <c r="A13" t="n">
         <v>2032</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>0</v>
       </c>
@@ -791,20 +710,12 @@
       <c r="A14" t="n">
         <v>2033</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>0</v>
       </c>
@@ -813,20 +724,12 @@
       <c r="A15" t="n">
         <v>2034</v>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -835,20 +738,12 @@
       <c r="A16" t="n">
         <v>2035</v>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
         <v>0</v>
       </c>
@@ -857,20 +752,12 @@
       <c r="A17" t="n">
         <v>2036</v>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>0</v>
       </c>
@@ -879,20 +766,12 @@
       <c r="A18" t="n">
         <v>2037</v>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>0</v>
       </c>
@@ -901,20 +780,12 @@
       <c r="A19" t="n">
         <v>2038</v>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="n">
         <v>0</v>
       </c>
@@ -923,20 +794,12 @@
       <c r="A20" t="n">
         <v>2039</v>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
         <v>0</v>
       </c>
@@ -945,20 +808,12 @@
       <c r="A21" t="n">
         <v>2040</v>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>0</v>
       </c>
@@ -967,20 +822,12 @@
       <c r="A22" t="n">
         <v>2041</v>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
         <v>0</v>
       </c>
@@ -989,20 +836,12 @@
       <c r="A23" t="n">
         <v>2042</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
         <v>0</v>
       </c>
@@ -1011,20 +850,12 @@
       <c r="A24" t="n">
         <v>2043</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
         <v>0</v>
       </c>
@@ -1033,20 +864,12 @@
       <c r="A25" t="n">
         <v>2044</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
         <v>0</v>
       </c>
@@ -1055,20 +878,12 @@
       <c r="A26" t="n">
         <v>2045</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
         <v>0</v>
       </c>
@@ -1077,20 +892,12 @@
       <c r="A27" t="n">
         <v>2046</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
         <v>0</v>
       </c>
@@ -1099,20 +906,12 @@
       <c r="A28" t="n">
         <v>2047</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
         <v>0</v>
       </c>
@@ -1121,20 +920,12 @@
       <c r="A29" t="n">
         <v>2048</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
         <v>0</v>
       </c>
@@ -1143,20 +934,12 @@
       <c r="A30" t="n">
         <v>2049</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
         <v>0</v>
       </c>
@@ -1165,20 +948,12 @@
       <c r="A31" t="n">
         <v>2050</v>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
         <v>0</v>
       </c>
@@ -1187,20 +962,12 @@
       <c r="A32" t="n">
         <v>2051</v>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
         <v>0</v>
       </c>
@@ -1209,20 +976,12 @@
       <c r="A33" t="n">
         <v>2052</v>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
         <v>0</v>
       </c>
@@ -1231,20 +990,12 @@
       <c r="A34" t="n">
         <v>2053</v>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="n">
         <v>0</v>
       </c>
@@ -1253,20 +1004,12 @@
       <c r="A35" t="n">
         <v>2054</v>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
         <v>0</v>
       </c>
@@ -1275,20 +1018,12 @@
       <c r="A36" t="n">
         <v>2055</v>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="n">
         <v>0</v>
       </c>
@@ -1373,22 +1108,15 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
         <v>4000</v>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>0</v>
       </c>
@@ -1397,22 +1125,15 @@
       <c r="A3" t="n">
         <v>2022</v>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>4000</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>0</v>
       </c>
@@ -1421,22 +1142,15 @@
       <c r="A4" t="n">
         <v>2023</v>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
         <v>4000</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>0</v>
       </c>
@@ -1454,15 +1168,9 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
         <v>12000</v>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>0</v>
       </c>
@@ -1480,15 +1188,9 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>5000</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>0</v>
       </c>
@@ -1506,13 +1208,6 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>4000</v>
       </c>
@@ -1530,13 +1225,6 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>4000</v>
       </c>
@@ -1554,13 +1242,6 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>0</v>
       </c>
@@ -1569,20 +1250,12 @@
       <c r="A10" t="n">
         <v>2029</v>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>0</v>
       </c>
@@ -1591,20 +1264,12 @@
       <c r="A11" t="n">
         <v>2030</v>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>0</v>
       </c>
@@ -1613,20 +1278,12 @@
       <c r="A12" t="n">
         <v>2031</v>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>0</v>
       </c>
@@ -1635,20 +1292,12 @@
       <c r="A13" t="n">
         <v>2032</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>0</v>
       </c>
@@ -1657,20 +1306,12 @@
       <c r="A14" t="n">
         <v>2033</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>0</v>
       </c>
@@ -1679,20 +1320,12 @@
       <c r="A15" t="n">
         <v>2034</v>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>0</v>
       </c>
@@ -1701,20 +1334,12 @@
       <c r="A16" t="n">
         <v>2035</v>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
         <v>0</v>
       </c>
@@ -1723,20 +1348,12 @@
       <c r="A17" t="n">
         <v>2036</v>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>0</v>
       </c>
@@ -1745,20 +1362,12 @@
       <c r="A18" t="n">
         <v>2037</v>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>0</v>
       </c>
@@ -1767,20 +1376,12 @@
       <c r="A19" t="n">
         <v>2038</v>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="n">
         <v>0</v>
       </c>
@@ -1789,20 +1390,12 @@
       <c r="A20" t="n">
         <v>2039</v>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
         <v>0</v>
       </c>
@@ -1811,20 +1404,12 @@
       <c r="A21" t="n">
         <v>2040</v>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>0</v>
       </c>
@@ -1833,20 +1418,12 @@
       <c r="A22" t="n">
         <v>2041</v>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
         <v>0</v>
       </c>
@@ -1855,20 +1432,12 @@
       <c r="A23" t="n">
         <v>2042</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
         <v>0</v>
       </c>
@@ -1877,20 +1446,12 @@
       <c r="A24" t="n">
         <v>2043</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
         <v>0</v>
       </c>
@@ -1899,20 +1460,12 @@
       <c r="A25" t="n">
         <v>2044</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
         <v>0</v>
       </c>
@@ -1921,20 +1474,12 @@
       <c r="A26" t="n">
         <v>2045</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
         <v>0</v>
       </c>
@@ -1943,20 +1488,12 @@
       <c r="A27" t="n">
         <v>2046</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
         <v>0</v>
       </c>
@@ -1965,20 +1502,12 @@
       <c r="A28" t="n">
         <v>2047</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
         <v>0</v>
       </c>
@@ -1987,20 +1516,12 @@
       <c r="A29" t="n">
         <v>2048</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
         <v>0</v>
       </c>
@@ -2009,20 +1530,12 @@
       <c r="A30" t="n">
         <v>2049</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
         <v>0</v>
       </c>
@@ -2031,20 +1544,12 @@
       <c r="A31" t="n">
         <v>2050</v>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
         <v>0</v>
       </c>
@@ -2053,20 +1558,12 @@
       <c r="A32" t="n">
         <v>2051</v>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
         <v>0</v>
       </c>
@@ -2075,20 +1572,12 @@
       <c r="A33" t="n">
         <v>2052</v>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
         <v>0</v>
       </c>
@@ -2097,20 +1586,12 @@
       <c r="A34" t="n">
         <v>2053</v>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="n">
         <v>0</v>
       </c>
@@ -2119,20 +1600,12 @@
       <c r="A35" t="n">
         <v>2054</v>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
         <v>0</v>
       </c>
@@ -2141,20 +1614,12 @@
       <c r="A36" t="n">
         <v>2055</v>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="n">
         <v>0</v>
       </c>
@@ -2163,20 +1628,12 @@
       <c r="A37" t="n">
         <v>2056</v>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
         <v>0</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="n">
         <v>0</v>
       </c>
@@ -2185,20 +1642,12 @@
       <c r="A38" t="n">
         <v>2057</v>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="n">
         <v>0</v>
       </c>
@@ -2207,20 +1656,12 @@
       <c r="A39" t="n">
         <v>2058</v>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="n">
         <v>0</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="n">
         <v>0</v>
       </c>
@@ -2388,7 +1829,7 @@
         <v>750000</v>
       </c>
       <c r="G2" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>

</xml_diff>